<commit_message>
filtro rival en Miclub -> informe de partido
</commit_message>
<xml_diff>
--- a/Matches.xlsx
+++ b/Matches.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29127"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7982797A-A556-44B2-95DE-774BC09E7E1D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CC065EB2-A312-409A-A361-324B1753E794}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -180,13 +180,11 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hipervínculo" xfId="1" builtinId="8"/>
@@ -474,7 +472,7 @@
     <col min="1" max="1" width="10.7109375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="10.7109375" customWidth="1"/>
     <col min="3" max="3" width="12" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="34.140625" customWidth="1"/>
+    <col min="4" max="4" width="29.7109375" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="17.5703125" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="14.7109375" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="19" bestFit="1" customWidth="1"/>
@@ -529,8 +527,8 @@
         <v>18</v>
       </c>
     </row>
-    <row r="2" spans="1:15" s="5" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="4">
+    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A2" s="2">
         <v>46071</v>
       </c>
       <c r="C2" s="2" t="str">
@@ -540,19 +538,19 @@
       <c r="D2" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="E2" s="5" t="s">
+      <c r="E2" t="s">
         <v>13</v>
       </c>
-      <c r="F2" s="5">
+      <c r="F2">
         <v>1</v>
       </c>
-      <c r="H2" s="5" t="s">
+      <c r="H2" t="s">
         <v>21</v>
       </c>
-      <c r="I2" s="5" t="s">
+      <c r="I2" t="s">
         <v>32</v>
       </c>
-      <c r="J2" s="5">
+      <c r="J2">
         <v>0</v>
       </c>
       <c r="K2" t="str">
@@ -563,13 +561,13 @@
         <f>CONCATENATE( "vs ",I2)</f>
         <v>vs J. Bellapampa</v>
       </c>
-      <c r="M2" s="5">
+      <c r="M2">
         <v>2</v>
       </c>
-      <c r="N2" s="5">
+      <c r="N2">
         <v>1</v>
       </c>
-      <c r="O2" s="5" t="s">
+      <c r="O2" t="s">
         <v>19</v>
       </c>
     </row>

</xml_diff>